<commit_message>
Refactor string handling in tools.py to remove comments and improve formatting, enhance note/title handling in helpers2, and update `write_table` calls with `y_pos` parameter.
</commit_message>
<xml_diff>
--- a/bccsu/reports/templates/template.xlsx
+++ b/bccsu/reports/templates/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26501"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camer\Documents\Projects\bccsu-tools\bccsu\reports\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cgrant\PycharmProjects\bccsu-tools\bccsu\reports\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83004BE-6414-402E-832A-CD35645C19B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5969B13C-CA6F-4B10-8058-AD7B1B5EC7D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Request" sheetId="42" r:id="rId1"/>
@@ -37,7 +37,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="9.5"/>
       <color rgb="FF112277"/>
@@ -247,7 +247,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="1">
@@ -423,7 +423,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4CF33C2-40E8-4BFA-B351-887890A98467}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>